<commit_message>
Reorganize R scripts and update malaria analyses, data, and plots
</commit_message>
<xml_diff>
--- a/R_Output/Table1_Agreement_Rankings.xlsx
+++ b/R_Output/Table1_Agreement_Rankings.xlsx
@@ -384,115 +384,115 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Temperature</t>
+          <t>Physicians per 1000 People</t>
         </is>
       </c>
       <c r="B2">
-        <v>0.215</v>
+        <v>0.103</v>
       </c>
       <c r="C2">
-        <v>0.209</v>
+        <v>0.113</v>
       </c>
       <c r="D2">
-        <v>-0.055</v>
+        <v>-0.066</v>
       </c>
       <c r="E2">
-        <v>-0.016</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Latitude</t>
+          <t>Rainfall</t>
         </is>
       </c>
       <c r="B3">
-        <v>0.196</v>
+        <v>0.095</v>
       </c>
       <c r="C3">
-        <v>0.185</v>
+        <v>0.144</v>
       </c>
       <c r="D3">
-        <v>0.037</v>
+        <v>0.179</v>
       </c>
       <c r="E3">
-        <v>0.079</v>
+        <v>0.131</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Physicians per 1000 People</t>
+          <t>Latitude</t>
         </is>
       </c>
       <c r="B4">
-        <v>0.15</v>
+        <v>0.066</v>
       </c>
       <c r="C4">
-        <v>0.155</v>
+        <v>0.067</v>
       </c>
       <c r="D4">
-        <v>-0.03</v>
+        <v>-0.05</v>
       </c>
       <c r="E4">
-        <v>0.006</v>
+        <v>-0.028</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rainfall</t>
+          <t>Population Age</t>
         </is>
       </c>
       <c r="B5">
-        <v>0.092</v>
+        <v>0.063</v>
       </c>
       <c r="C5">
-        <v>0.131</v>
+        <v>0.052</v>
       </c>
       <c r="D5">
-        <v>0.15</v>
+        <v>-0.029</v>
       </c>
       <c r="E5">
-        <v>0.127</v>
+        <v>-0.006</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Population Age</t>
+          <t>Population Density</t>
         </is>
       </c>
       <c r="B6">
-        <v>0.08599999999999999</v>
+        <v>0.018</v>
       </c>
       <c r="C6">
-        <v>0.064</v>
+        <v>0.001</v>
       </c>
       <c r="D6">
-        <v>-0.034</v>
+        <v>-0.053</v>
       </c>
       <c r="E6">
-        <v>-0.005</v>
+        <v>-0.021</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Elevation</t>
+          <t>Temperature</t>
         </is>
       </c>
       <c r="B7">
-        <v>0.057</v>
+        <v>0.015</v>
       </c>
       <c r="C7">
-        <v>0.045</v>
+        <v>0.006</v>
       </c>
       <c r="D7">
-        <v>-0.064</v>
+        <v>-0.044</v>
       </c>
       <c r="E7">
-        <v>-0.046</v>
+        <v>-0.039</v>
       </c>
     </row>
     <row r="8">
@@ -502,35 +502,35 @@
         </is>
       </c>
       <c r="B8">
-        <v>0.045</v>
+        <v>0.011</v>
       </c>
       <c r="C8">
-        <v>0.08400000000000001</v>
+        <v>0.044</v>
       </c>
       <c r="D8">
-        <v>-0.044</v>
+        <v>-0.046</v>
       </c>
       <c r="E8">
-        <v>-0.014</v>
+        <v>-0.032</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Population Density</t>
+          <t>Elevation</t>
         </is>
       </c>
       <c r="B9">
-        <v>0.015</v>
+        <v>-0.003</v>
       </c>
       <c r="C9">
-        <v>-0.006</v>
+        <v>0.003</v>
       </c>
       <c r="D9">
-        <v>-0.052</v>
+        <v>-0.08</v>
       </c>
       <c r="E9">
-        <v>-0.023</v>
+        <v>-0.066</v>
       </c>
     </row>
   </sheetData>

</xml_diff>